<commit_message>
App entrevista: emparejamiento automatico avatar/voz + migracion a Anam (voces ES, fix llmId)
</commit_message>
<xml_diff>
--- a/resultados experimentos/DAM_por_pregunta_Barometro_Digital.xlsx
+++ b/resultados experimentos/DAM_por_pregunta_Barometro_Digital.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://deusto-my.sharepoint.com/personal/druiz_deusto_es/Documents/Documentos/claude/Projects/Pueblo digital/resultados experimentos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_A1D0FEDB9FF8230488CADC72E9B661A450139458" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C060FCAA-6C0D-434A-BE60-FB37737EE1CF}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="11_A1D0FEDB9FF8230488CADC72E9B661A450139458" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E05E4037-72D6-495E-8E76-0E0643D6DDBC}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" tabRatio="726" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="726" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Detalle por pregunta" sheetId="1" r:id="rId1"/>
@@ -35,6 +35,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -43,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="357">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="365">
   <si>
     <t>Bloque</t>
   </si>
@@ -1114,6 +1117,30 @@
   </si>
   <si>
     <t>¿Cuál de las frases que aparecen en esta tarjeta describe mejor el lugar donde vive?</t>
+  </si>
+  <si>
+    <t>Llave</t>
+  </si>
+  <si>
+    <t>ciudad</t>
+  </si>
+  <si>
+    <t>sexo</t>
+  </si>
+  <si>
+    <t>educación</t>
+  </si>
+  <si>
+    <t>situación laboral</t>
+  </si>
+  <si>
+    <t>provincia</t>
+  </si>
+  <si>
+    <t>clase</t>
+  </si>
+  <si>
+    <t>ideología</t>
   </si>
 </sst>
 </file>
@@ -1123,7 +1150,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1173,6 +1200,13 @@
     <font>
       <sz val="9"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
@@ -1286,7 +1320,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1370,6 +1404,7 @@
     <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -4545,7 +4580,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6439460F-18AC-4019-A68B-9205B2CDBF85}">
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43" style="18" customWidth="1"/>
@@ -4555,9 +4590,10 @@
     <col min="5" max="5" width="30.28515625" style="18" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="2.28515625" customWidth="1"/>
     <col min="7" max="7" width="19.5703125" customWidth="1"/>
+    <col min="8" max="8" width="2.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>323</v>
       </c>
@@ -4574,8 +4610,11 @@
         <v>355</v>
       </c>
       <c r="H1" s="21"/>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="20" t="s">
         <v>320</v>
       </c>
@@ -4588,7 +4627,7 @@
       <c r="F2" s="22"/>
       <c r="G2" s="22"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="20" t="s">
         <v>321</v>
       </c>
@@ -4601,7 +4640,7 @@
       <c r="F3" s="22"/>
       <c r="G3" s="22"/>
     </row>
-    <row r="4" spans="1:8" ht="24.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" ht="24.75" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>337</v>
       </c>
@@ -4614,7 +4653,7 @@
       <c r="F4" s="22"/>
       <c r="G4" s="22"/>
     </row>
-    <row r="5" spans="1:8" ht="24.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" ht="24.75" x14ac:dyDescent="0.25">
       <c r="C5" s="20" t="s">
         <v>347</v>
       </c>
@@ -4622,7 +4661,7 @@
       <c r="E5" s="20"/>
       <c r="F5" s="22"/>
     </row>
-    <row r="6" spans="1:8" ht="48.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" ht="48.75" x14ac:dyDescent="0.25">
       <c r="A6" s="25" t="s">
         <v>338</v>
       </c>
@@ -4638,8 +4677,11 @@
       <c r="G6" s="25" t="s">
         <v>356</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I6" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="26" t="s">
         <v>322</v>
       </c>
@@ -4655,8 +4697,11 @@
       <c r="G7" s="26" t="s">
         <v>329</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" ht="24.75" x14ac:dyDescent="0.25">
+      <c r="I7" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="24.75" x14ac:dyDescent="0.25">
       <c r="A8" s="27" t="s">
         <v>339</v>
       </c>
@@ -4673,7 +4718,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="36.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" ht="36.75" x14ac:dyDescent="0.25">
       <c r="A9" s="28" t="s">
         <v>340</v>
       </c>
@@ -4689,8 +4734,11 @@
       <c r="G9" s="28" t="s">
         <v>350</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" ht="24.75" x14ac:dyDescent="0.25">
+      <c r="I9" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="24.75" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
         <v>341</v>
       </c>
@@ -4701,7 +4749,7 @@
       </c>
       <c r="F10" s="22"/>
     </row>
-    <row r="11" spans="1:8" ht="24.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" ht="24.75" x14ac:dyDescent="0.25">
       <c r="A11" s="20" t="s">
         <v>342</v>
       </c>
@@ -4710,13 +4758,10 @@
         <v>351</v>
       </c>
       <c r="D11" s="22"/>
-      <c r="E11" s="20" t="s">
-        <v>333</v>
-      </c>
       <c r="F11" s="22"/>
       <c r="G11" s="22"/>
     </row>
-    <row r="12" spans="1:8" ht="24.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" ht="24.75" x14ac:dyDescent="0.25">
       <c r="A12" s="23" t="s">
         <v>343</v>
       </c>
@@ -4732,8 +4777,11 @@
       <c r="G12" s="23" t="s">
         <v>334</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I12" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="29" t="s">
         <v>344</v>
       </c>
@@ -4747,14 +4795,28 @@
       </c>
       <c r="F13" s="22"/>
       <c r="G13" s="22"/>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I13" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="20" t="s">
         <v>345</v>
       </c>
       <c r="B14" s="20"/>
       <c r="C14" s="20" t="s">
         <v>354</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>333</v>
+      </c>
+      <c r="I14" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I15" s="31" t="s">
+        <v>364</v>
       </c>
     </row>
   </sheetData>

</xml_diff>